<commit_message>
primeira estrat: precisa melhorar rebalenceamento, mov. avg, ...
</commit_message>
<xml_diff>
--- a/etfs.xlsx
+++ b/etfs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tomasrolimmiele/Desktop/Insper - Eng. Comp/8o Sem/Capstone/202601_PG_Modelagem_Preditiva/databases/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tomasrolimmiele/Desktop/Insper - Eng. Comp/8o Sem/Eng Analytics VI/etf_strategy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14838E14-CD8C-4F4B-BF08-E652DC1904FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64467023-5FAF-7B43-A8BF-C918E48D8B15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{30C33318-D82E-5243-966F-BE490FF6293F}"/>
   </bookViews>
@@ -41,9 +41,6 @@
     <t>Country</t>
   </si>
   <si>
-    <t>Code</t>
-  </si>
-  <si>
     <t>Brazil</t>
   </si>
   <si>
@@ -168,6 +165,9 @@
   </si>
   <si>
     <t>THD</t>
+  </si>
+  <si>
+    <t>Ticker</t>
   </si>
 </sst>
 </file>
@@ -556,175 +556,175 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
         <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
         <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
         <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
         <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
         <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
         <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
         <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
         <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
         <v>20</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
         <v>22</v>
-      </c>
-      <c r="B12" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" t="s">
         <v>24</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" t="s">
         <v>26</v>
-      </c>
-      <c r="B14" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" t="s">
         <v>28</v>
-      </c>
-      <c r="B15" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" t="s">
         <v>30</v>
-      </c>
-      <c r="B16" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" t="s">
         <v>32</v>
-      </c>
-      <c r="B17" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" t="s">
         <v>34</v>
-      </c>
-      <c r="B18" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" t="s">
         <v>36</v>
-      </c>
-      <c r="B19" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>37</v>
+      </c>
+      <c r="B20" t="s">
         <v>38</v>
-      </c>
-      <c r="B20" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" t="s">
         <v>40</v>
-      </c>
-      <c r="B21" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22" t="s">
         <v>42</v>
-      </c>
-      <c r="B22" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>